<commit_message>
Log US/EU/Asia TOPIC_SELECTED entries for run MA-CF-20260916-094234
Registers the three real-mode selections made during today's Content
Factory run (FOMC, ECB, BOJ) for cross-run duplicate detection.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/content-log/selected-topics.xlsx
+++ b/data/content-log/selected-topics.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="59">
   <si>
     <t>run_id</t>
   </si>
@@ -122,6 +122,72 @@
   </si>
   <si>
     <t>Explaining the BOJ's exit mechanism from ultra-easy policy and its yen/portfolio implications</t>
+  </si>
+  <si>
+    <t>MA-CF-20260916-094234</t>
+  </si>
+  <si>
+    <t>MA-CF-20260916-094234-US</t>
+  </si>
+  <si>
+    <t>2026-09-16T10:05:53Z</t>
+  </si>
+  <si>
+    <t>US-FOMC-20260916</t>
+  </si>
+  <si>
+    <t>FOMC September 2026 Rate Decision: Reading the Vote, the Dot Plot, and Chair Warsh's Signal</t>
+  </si>
+  <si>
+    <t>IMMEDIATE</t>
+  </si>
+  <si>
+    <t>Fed, FOMC, Interest Rates, Kevin Warsh, Dot Plot</t>
+  </si>
+  <si>
+    <t>Decompose the vote count, updated rate projections (dot plot), and Chair Warsh's press-conference tone rather than reporting the headline decision alone.</t>
+  </si>
+  <si>
+    <t>real</t>
+  </si>
+  <si>
+    <t>MA-CF-20260916-094234-EUROPE</t>
+  </si>
+  <si>
+    <t>EUROPE</t>
+  </si>
+  <si>
+    <t>EU-ECB-20260916</t>
+  </si>
+  <si>
+    <t>ECB Raises Rates to 2.50% as Middle East Conflict Drives Inflation Pressure</t>
+  </si>
+  <si>
+    <t>92</t>
+  </si>
+  <si>
+    <t>ECB, Interest Rates, Inflation, Middle East Conflict, Energy Prices</t>
+  </si>
+  <si>
+    <t>Explain the transmission mechanism from Middle East conflict-driven energy inflation to the ECB's second 2026 hike and its projected disinflation path through 2028.</t>
+  </si>
+  <si>
+    <t>MA-CF-20260916-094234-ASIA</t>
+  </si>
+  <si>
+    <t>ASIA-BOJ-20260918</t>
+  </si>
+  <si>
+    <t>Bank of Japan's September Meeting: What a Near-Unanimous Hike Call Means for the Normalization Path</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>Bank of Japan, BOJ, Interest Rates, Yen, Monetary Policy Normalization</t>
+  </si>
+  <si>
+    <t>Explain what is at stake in the BOJ's near-unanimously expected hike and the normalization path ahead, without presuming the outcome before it is announced.</t>
   </si>
 </sst>
 </file>
@@ -502,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="18" customWidth="1"/>
@@ -645,6 +711,138 @@
         <v>26</v>
       </c>
     </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" t="s">
+        <v>43</v>
+      </c>
+      <c r="L4" t="s">
+        <v>44</v>
+      </c>
+      <c r="M4" t="s">
+        <v>45</v>
+      </c>
+      <c r="N4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M5" t="s">
+        <v>45</v>
+      </c>
+      <c r="N5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" t="s">
+        <v>57</v>
+      </c>
+      <c r="L6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M6" t="s">
+        <v>45</v>
+      </c>
+      <c r="N6" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>